<commit_message>
add Alternatif management feature with model, migration, Livewire component, and view; update Balita model and routes
</commit_message>
<xml_diff>
--- a/public/lhfa_0-to-5-years_zscores.xlsx
+++ b/public/lhfa_0-to-5-years_zscores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yry\Desktop\SKRIPSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A77F2D3-A21A-4976-9558-B0CFFE3179D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AEEB57-A23B-43BC-B662-D7D8C996FF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,12 +21,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="13">
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
   <si>
     <t>month</t>
   </si>
@@ -59,6 +53,12 @@
   </si>
   <si>
     <t>plus_3sd</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
 </sst>
 </file>
@@ -942,37 +942,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
-      </c>
-      <c r="J1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -980,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>49.1477</v>
@@ -1015,7 +1015,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>53.687199999999997</v>
@@ -1050,7 +1050,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>57.067300000000003</v>
@@ -1085,7 +1085,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>59.802900000000001</v>
@@ -1120,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>62.0899</v>
@@ -1155,7 +1155,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C7">
         <v>64.030100000000004</v>
@@ -1190,7 +1190,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C8">
         <v>65.731099999999998</v>
@@ -1225,7 +1225,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C9">
         <v>67.287300000000002</v>
@@ -1260,7 +1260,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C10">
         <v>68.749799999999993</v>
@@ -1295,7 +1295,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C11">
         <v>70.143500000000003</v>
@@ -1330,7 +1330,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C12">
         <v>71.481800000000007</v>
@@ -1365,7 +1365,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C13">
         <v>72.771000000000001</v>
@@ -1400,7 +1400,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C14">
         <v>74.015000000000001</v>
@@ -1435,7 +1435,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C15">
         <v>75.217600000000004</v>
@@ -1470,7 +1470,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C16">
         <v>76.381699999999995</v>
@@ -1505,7 +1505,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C17">
         <v>77.509900000000002</v>
@@ -1540,7 +1540,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C18">
         <v>78.605500000000006</v>
@@ -1575,7 +1575,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C19">
         <v>79.671000000000006</v>
@@ -1610,7 +1610,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C20">
         <v>80.707899999999995</v>
@@ -1645,7 +1645,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C21">
         <v>81.718199999999996</v>
@@ -1680,7 +1680,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C22">
         <v>82.703599999999994</v>
@@ -1715,7 +1715,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C23">
         <v>83.665400000000005</v>
@@ -1750,7 +1750,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C24">
         <v>84.603999999999999</v>
@@ -1785,7 +1785,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C25">
         <v>85.520200000000003</v>
@@ -1820,7 +1820,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C26">
         <v>85.715299999999999</v>
@@ -1855,7 +1855,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C27">
         <v>86.590400000000002</v>
@@ -1890,7 +1890,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C28">
         <v>87.446200000000005</v>
@@ -1925,7 +1925,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C29">
         <v>88.283000000000001</v>
@@ -1960,7 +1960,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C30">
         <v>89.100399999999993</v>
@@ -1995,7 +1995,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C31">
         <v>89.899100000000004</v>
@@ -2030,7 +2030,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C32">
         <v>90.679699999999997</v>
@@ -2065,7 +2065,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C33">
         <v>91.442999999999998</v>
@@ -2100,7 +2100,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C34">
         <v>92.190600000000003</v>
@@ -2135,7 +2135,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C35">
         <v>92.923900000000003</v>
@@ -2170,7 +2170,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C36">
         <v>93.644400000000005</v>
@@ -2205,7 +2205,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C37">
         <v>94.353300000000004</v>
@@ -2240,7 +2240,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C38">
         <v>95.051500000000004</v>
@@ -2275,7 +2275,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C39">
         <v>95.739900000000006</v>
@@ -2310,7 +2310,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C40">
         <v>96.418700000000001</v>
@@ -2345,7 +2345,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C41">
         <v>97.088499999999996</v>
@@ -2380,7 +2380,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C42">
         <v>97.749300000000005</v>
@@ -2415,7 +2415,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C43">
         <v>98.401499999999999</v>
@@ -2450,7 +2450,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C44">
         <v>99.044799999999995</v>
@@ -2485,7 +2485,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C45">
         <v>99.679500000000004</v>
@@ -2520,7 +2520,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C46">
         <v>100.3058</v>
@@ -2555,7 +2555,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C47">
         <v>100.9238</v>
@@ -2590,7 +2590,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C48">
         <v>101.5337</v>
@@ -2625,7 +2625,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C49">
         <v>102.136</v>
@@ -2660,7 +2660,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C50">
         <v>102.7312</v>
@@ -2695,7 +2695,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C51">
         <v>103.3197</v>
@@ -2730,7 +2730,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C52">
         <v>103.9021</v>
@@ -2765,7 +2765,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C53">
         <v>104.4786</v>
@@ -2800,7 +2800,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C54">
         <v>105.04940000000001</v>
@@ -2835,7 +2835,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C55">
         <v>105.6148</v>
@@ -2870,7 +2870,7 @@
         <v>54</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C56">
         <v>106.1748</v>
@@ -2905,7 +2905,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C57">
         <v>106.7295</v>
@@ -2940,7 +2940,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C58">
         <v>107.2788</v>
@@ -2975,7 +2975,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C59">
         <v>107.8227</v>
@@ -3010,7 +3010,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C60">
         <v>108.3613</v>
@@ -3045,7 +3045,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C61">
         <v>108.8948</v>
@@ -3080,7 +3080,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C62">
         <v>109.4233</v>
@@ -3115,7 +3115,7 @@
         <v>0</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C63">
         <v>49.8842</v>
@@ -3150,7 +3150,7 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C64">
         <v>54.724400000000003</v>
@@ -3185,7 +3185,7 @@
         <v>2</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C65">
         <v>58.424900000000001</v>
@@ -3220,7 +3220,7 @@
         <v>3</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C66">
         <v>61.429200000000002</v>
@@ -3255,7 +3255,7 @@
         <v>4</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C67">
         <v>63.886000000000003</v>
@@ -3290,7 +3290,7 @@
         <v>5</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C68">
         <v>65.902600000000007</v>
@@ -3325,7 +3325,7 @@
         <v>6</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C69">
         <v>67.623599999999996</v>
@@ -3360,7 +3360,7 @@
         <v>7</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C70">
         <v>69.164500000000004</v>
@@ -3395,7 +3395,7 @@
         <v>8</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C71">
         <v>70.599400000000003</v>
@@ -3430,7 +3430,7 @@
         <v>9</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C72">
         <v>71.968699999999998</v>
@@ -3465,7 +3465,7 @@
         <v>10</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C73">
         <v>73.281199999999998</v>
@@ -3500,7 +3500,7 @@
         <v>11</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C74">
         <v>74.538799999999995</v>
@@ -3535,7 +3535,7 @@
         <v>12</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C75">
         <v>75.748800000000003</v>
@@ -3570,7 +3570,7 @@
         <v>13</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C76">
         <v>76.918599999999998</v>
@@ -3605,7 +3605,7 @@
         <v>14</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C77">
         <v>78.049700000000001</v>
@@ -3640,7 +3640,7 @@
         <v>15</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C78">
         <v>79.145799999999994</v>
@@ -3675,7 +3675,7 @@
         <v>16</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C79">
         <v>80.211299999999994</v>
@@ -3710,7 +3710,7 @@
         <v>17</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C80">
         <v>81.248699999999999</v>
@@ -3745,7 +3745,7 @@
         <v>18</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C81">
         <v>82.258700000000005</v>
@@ -3780,7 +3780,7 @@
         <v>19</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C82">
         <v>83.241799999999998</v>
@@ -3815,7 +3815,7 @@
         <v>20</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C83">
         <v>84.199600000000004</v>
@@ -3850,7 +3850,7 @@
         <v>21</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C84">
         <v>85.134799999999998</v>
@@ -3885,7 +3885,7 @@
         <v>22</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C85">
         <v>86.047700000000006</v>
@@ -3920,7 +3920,7 @@
         <v>23</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C86">
         <v>86.941000000000003</v>
@@ -3955,7 +3955,7 @@
         <v>24</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C87">
         <v>87.116100000000003</v>
@@ -3990,7 +3990,7 @@
         <v>25</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C88">
         <v>87.971999999999994</v>
@@ -4025,7 +4025,7 @@
         <v>26</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C89">
         <v>88.8065</v>
@@ -4060,7 +4060,7 @@
         <v>27</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C90">
         <v>89.619699999999995</v>
@@ -4095,7 +4095,7 @@
         <v>28</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C91">
         <v>90.412000000000006</v>
@@ -4130,7 +4130,7 @@
         <v>29</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C92">
         <v>91.1828</v>
@@ -4165,7 +4165,7 @@
         <v>30</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C93">
         <v>91.932699999999997</v>
@@ -4200,7 +4200,7 @@
         <v>31</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C94">
         <v>92.6631</v>
@@ -4235,7 +4235,7 @@
         <v>32</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C95">
         <v>93.375299999999996</v>
@@ -4270,7 +4270,7 @@
         <v>33</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C96">
         <v>94.071100000000001</v>
@@ -4305,7 +4305,7 @@
         <v>34</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C97">
         <v>94.753200000000007</v>
@@ -4340,7 +4340,7 @@
         <v>35</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C98">
         <v>95.423599999999993</v>
@@ -4375,7 +4375,7 @@
         <v>36</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C99">
         <v>96.083500000000001</v>
@@ -4410,7 +4410,7 @@
         <v>37</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C100">
         <v>96.733699999999999</v>
@@ -4445,7 +4445,7 @@
         <v>38</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C101">
         <v>97.374899999999997</v>
@@ -4480,7 +4480,7 @@
         <v>39</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C102">
         <v>98.007300000000001</v>
@@ -4515,7 +4515,7 @@
         <v>40</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C103">
         <v>98.631</v>
@@ -4550,7 +4550,7 @@
         <v>41</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C104">
         <v>99.245900000000006</v>
@@ -4585,7 +4585,7 @@
         <v>42</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C105">
         <v>99.851500000000001</v>
@@ -4620,7 +4620,7 @@
         <v>43</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C106">
         <v>100.4485</v>
@@ -4655,7 +4655,7 @@
         <v>44</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C107">
         <v>101.03740000000001</v>
@@ -4690,7 +4690,7 @@
         <v>45</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C108">
         <v>101.6186</v>
@@ -4725,7 +4725,7 @@
         <v>46</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C109">
         <v>102.19329999999999</v>
@@ -4760,7 +4760,7 @@
         <v>47</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C110">
         <v>102.7625</v>
@@ -4795,7 +4795,7 @@
         <v>48</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C111">
         <v>103.32729999999999</v>
@@ -4830,7 +4830,7 @@
         <v>49</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C112">
         <v>103.8886</v>
@@ -4865,7 +4865,7 @@
         <v>50</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C113">
         <v>104.4473</v>
@@ -4900,7 +4900,7 @@
         <v>51</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C114">
         <v>105.00409999999999</v>
@@ -4935,7 +4935,7 @@
         <v>52</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C115">
         <v>105.5596</v>
@@ -4970,7 +4970,7 @@
         <v>53</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C116">
         <v>106.1138</v>
@@ -5005,7 +5005,7 @@
         <v>54</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C117">
         <v>106.66679999999999</v>
@@ -5040,7 +5040,7 @@
         <v>55</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C118">
         <v>107.2188</v>
@@ -5075,7 +5075,7 @@
         <v>56</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C119">
         <v>107.7697</v>
@@ -5110,7 +5110,7 @@
         <v>57</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C120">
         <v>108.3198</v>
@@ -5145,7 +5145,7 @@
         <v>58</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C121">
         <v>108.8689</v>
@@ -5180,7 +5180,7 @@
         <v>59</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C122">
         <v>109.417</v>
@@ -5215,7 +5215,7 @@
         <v>60</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C123">
         <v>109.96380000000001</v>

</xml_diff>